<commit_message>
added ports to bjts, passives, via stack
</commit_message>
<xml_diff>
--- a/Klayout PyCell Checklist.xlsx
+++ b/Klayout PyCell Checklist.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="45">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -58,6 +58,9 @@
     <t xml:space="preserve">bondpads</t>
   </si>
   <si>
+    <t xml:space="preserve">wie?</t>
+  </si>
+  <si>
     <t xml:space="preserve">cmim</t>
   </si>
   <si>
@@ -122,9 +125,6 @@
   </si>
   <si>
     <t xml:space="preserve">rfcmim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rfmosfet_base</t>
   </si>
   <si>
     <t xml:space="preserve">rfnmos</t>
@@ -468,12 +468,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr defaultColWidth="11.5390625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16.05"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.03"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="12.11"/>
   </cols>
   <sheetData>
@@ -539,11 +539,13 @@
       <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="3"/>
+      <c r="E4" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>9</v>
@@ -558,10 +560,10 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>7</v>
@@ -573,10 +575,10 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>7</v>
@@ -588,10 +590,10 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>7</v>
@@ -599,14 +601,16 @@
       <c r="D8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="3"/>
+      <c r="E8" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>7</v>
@@ -618,10 +622,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>7</v>
@@ -633,10 +637,10 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>7</v>
@@ -648,10 +652,10 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>23</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>22</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>7</v>
@@ -663,10 +667,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>7</v>
@@ -674,29 +678,33 @@
       <c r="D13" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E13" s="3"/>
+      <c r="E13" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="C14" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E14" s="3"/>
+      <c r="E14" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>7</v>
@@ -704,14 +712,16 @@
       <c r="D15" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E15" s="3"/>
+      <c r="E15" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>7</v>
@@ -719,14 +729,16 @@
       <c r="D16" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E16" s="3"/>
+      <c r="E16" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>7</v>
@@ -738,10 +750,10 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>7</v>
@@ -753,10 +765,10 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>7</v>
@@ -764,14 +776,16 @@
       <c r="D19" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E19" s="3"/>
+      <c r="E19" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>7</v>
@@ -779,11 +793,13 @@
       <c r="D20" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="3"/>
+      <c r="E20" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>9</v>
@@ -798,21 +814,25 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
+        <v>23</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>7</v>
+      </c>
       <c r="E22" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>7</v>
@@ -824,10 +844,10 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>7</v>
@@ -839,10 +859,10 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>7</v>
@@ -854,10 +874,10 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>7</v>
@@ -869,7 +889,7 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>40</v>
@@ -884,7 +904,7 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>40</v>
@@ -899,10 +919,10 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="C29" s="3" t="s">
         <v>7</v>
@@ -910,14 +930,16 @@
       <c r="D29" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E29" s="3"/>
+      <c r="E29" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>7</v>
@@ -925,25 +947,12 @@
       <c r="D30" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E30" s="3"/>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E31" s="3"/>
+      <c r="E30" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="C2:E31">
+  <conditionalFormatting sqref="C2:E30">
     <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="y" dxfId="0">
       <formula>NOT(ISERROR(SEARCH("y",C2)))</formula>
     </cfRule>

</xml_diff>

<commit_message>
added ports to capacitors
</commit_message>
<xml_diff>
--- a/Klayout PyCell Checklist.xlsx
+++ b/Klayout PyCell Checklist.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="45">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -524,7 +524,9 @@
       <c r="D3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
@@ -556,7 +558,9 @@
       <c r="D5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E5" s="3"/>
+      <c r="E5" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
@@ -571,7 +575,9 @@
       <c r="D6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E6" s="3"/>
+      <c r="E6" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
@@ -586,7 +592,9 @@
       <c r="D7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="3"/>
+      <c r="E7" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
@@ -618,7 +626,9 @@
       <c r="D9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="3"/>
+      <c r="E9" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
@@ -633,7 +643,9 @@
       <c r="D10" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E10" s="3"/>
+      <c r="E10" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
@@ -810,7 +822,9 @@
       <c r="D21" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E21" s="3"/>
+      <c r="E21" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
@@ -885,7 +899,9 @@
       <c r="D26" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E26" s="3"/>
+      <c r="E26" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
@@ -900,7 +916,9 @@
       <c r="D27" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E27" s="3"/>
+      <c r="E27" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
@@ -915,7 +933,9 @@
       <c r="D28" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E28" s="3"/>
+      <c r="E28" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">

</xml_diff>

<commit_message>
Update Klayout PyCell Checklist.xlsx
</commit_message>
<xml_diff>
--- a/Klayout PyCell Checklist.xlsx
+++ b/Klayout PyCell Checklist.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="45">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -660,7 +660,9 @@
       <c r="D11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="3"/>
+      <c r="E11" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
@@ -675,7 +677,9 @@
       <c r="D12" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="3"/>
+      <c r="E12" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
@@ -758,7 +762,9 @@
       <c r="D17" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E17" s="3"/>
+      <c r="E17" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
@@ -773,7 +779,9 @@
       <c r="D18" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="3"/>
+      <c r="E18" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">

</xml_diff>